<commit_message>
Update: finalizada práctica final de curso básico
</commit_message>
<xml_diff>
--- a/excel/08 - BD PERSONAS.xlsx
+++ b/excel/08 - BD PERSONAS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://formabyte-my.sharepoint.com/personal/econdor_formabyte_onmicrosoft_com/Documents/CLIENTES/GLOBAL ALUMINI (Empresa Nachete)/CURSO POWER BI/FICHEROS A ADJUNTAR EN EL CURSO/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/632c24d3e29ca445/Desktop/Excel-Power-Analytics/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{04F5EAFD-AEE2-4788-BB0C-6E3756EDB910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D35DD4F-A3CD-4CA1-88ED-821A9759FBF3}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{04F5EAFD-AEE2-4788-BB0C-6E3756EDB910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF4F8FDA-D5B3-4E9F-8F09-6DDC0DDFE8D3}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{54C4B625-833A-4851-811C-E766E7ECB1A5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{54C4B625-833A-4851-811C-E766E7ECB1A5}"/>
   </bookViews>
   <sheets>
     <sheet name="CLIENTES" sheetId="1" r:id="rId1"/>
@@ -1069,7 +1069,30 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1080,6 +1103,21 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DF8A5B36-A3BE-44E2-8E3E-F747363A173C}" name="T_CLIENTE" displayName="T_CLIENTE" ref="A1:F115" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:F115" xr:uid="{DF8A5B36-A3BE-44E2-8E3E-F747363A173C}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{7E72E293-6729-4907-AC63-4322C85AE93B}" name="COD CLIENTE"/>
+    <tableColumn id="2" xr3:uid="{C0D9D3CD-0672-43FD-8A47-717E90658628}" name="NOMBRE"/>
+    <tableColumn id="3" xr3:uid="{C855A4F5-8288-425E-85F1-1011B40C8E8E}" name="APELLIDO1"/>
+    <tableColumn id="4" xr3:uid="{3C640ACD-8943-4A70-882E-D5BC0195434D}" name="APELLIDO 2"/>
+    <tableColumn id="5" xr3:uid="{E1A1B30E-9633-4BA1-BA53-30C99E2067F1}" name="NIF"/>
+    <tableColumn id="6" xr3:uid="{2064C436-16DB-4858-B4C3-97EDC17954E5}" name="FECHA INCORPORACION" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1380,16 +1418,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8CB2FEA-898C-4607-B7B5-E16D48D02E7C}">
   <dimension ref="A1:F115"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5546875" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="5" width="10.88671875" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.5546875" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1409,7 +1447,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1968</v>
       </c>
@@ -1429,7 +1467,7 @@
         <v>43652</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1674</v>
       </c>
@@ -1449,7 +1487,7 @@
         <v>44429</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1516</v>
       </c>
@@ -1469,7 +1507,7 @@
         <v>44320</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1330</v>
       </c>
@@ -1489,7 +1527,7 @@
         <v>43625</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1657</v>
       </c>
@@ -1509,7 +1547,7 @@
         <v>43746</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1573</v>
       </c>
@@ -1529,7 +1567,7 @@
         <v>43933</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1658</v>
       </c>
@@ -1549,7 +1587,7 @@
         <v>44382</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1078</v>
       </c>
@@ -1569,7 +1607,7 @@
         <v>43907</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1695</v>
       </c>
@@ -1589,7 +1627,7 @@
         <v>43808</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>1285</v>
       </c>
@@ -1609,7 +1647,7 @@
         <v>44009</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>1284</v>
       </c>
@@ -1629,7 +1667,7 @@
         <v>43780</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>1517</v>
       </c>
@@ -1649,7 +1687,7 @@
         <v>44429</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>1674</v>
       </c>
@@ -1669,7 +1707,7 @@
         <v>44032</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>1056</v>
       </c>
@@ -1689,7 +1727,7 @@
         <v>44280</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>1977</v>
       </c>
@@ -1709,7 +1747,7 @@
         <v>44293</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>1725</v>
       </c>
@@ -1729,7 +1767,7 @@
         <v>44252</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>1675</v>
       </c>
@@ -1749,7 +1787,7 @@
         <v>43949</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>1968</v>
       </c>
@@ -1769,7 +1807,7 @@
         <v>44225</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>1723</v>
       </c>
@@ -1789,7 +1827,7 @@
         <v>44008</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>1076</v>
       </c>
@@ -1809,7 +1847,7 @@
         <v>43576</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>1816</v>
       </c>
@@ -1829,7 +1867,7 @@
         <v>43843</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>1154</v>
       </c>
@@ -1849,7 +1887,7 @@
         <v>44312</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>1294</v>
       </c>
@@ -1869,7 +1907,7 @@
         <v>43890</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>1428</v>
       </c>
@@ -1889,7 +1927,7 @@
         <v>43592</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>1814</v>
       </c>
@@ -1909,7 +1947,7 @@
         <v>44064</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>1978</v>
       </c>
@@ -1929,7 +1967,7 @@
         <v>43615</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>1531</v>
       </c>
@@ -1949,7 +1987,7 @@
         <v>44428</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>1931</v>
       </c>
@@ -1969,7 +2007,7 @@
         <v>44015</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>1932</v>
       </c>
@@ -1989,7 +2027,7 @@
         <v>43929</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>1291</v>
       </c>
@@ -2009,7 +2047,7 @@
         <v>43609</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>1530</v>
       </c>
@@ -2029,7 +2067,7 @@
         <v>44172</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>1152</v>
       </c>
@@ -2049,7 +2087,7 @@
         <v>43966</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>1079</v>
       </c>
@@ -2069,7 +2107,7 @@
         <v>43614</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>1676</v>
       </c>
@@ -2089,7 +2127,7 @@
         <v>44210</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>1290</v>
       </c>
@@ -2109,7 +2147,7 @@
         <v>43808</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>1961</v>
       </c>
@@ -2129,7 +2167,7 @@
         <v>43692</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>1675</v>
       </c>
@@ -2149,7 +2187,7 @@
         <v>44349</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>1368</v>
       </c>
@@ -2169,7 +2207,7 @@
         <v>43922</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>1153</v>
       </c>
@@ -2189,7 +2227,7 @@
         <v>44019</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>1960</v>
       </c>
@@ -2209,7 +2247,7 @@
         <v>44236</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>1908</v>
       </c>
@@ -2229,7 +2267,7 @@
         <v>43493</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>1011</v>
       </c>
@@ -2249,7 +2287,7 @@
         <v>44324</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>1359</v>
       </c>
@@ -2269,7 +2307,7 @@
         <v>43941</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>1724</v>
       </c>
@@ -2289,7 +2327,7 @@
         <v>43512</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>1923</v>
       </c>
@@ -2309,7 +2347,7 @@
         <v>44016</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>1794</v>
       </c>
@@ -2329,7 +2367,7 @@
         <v>43812</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>1558</v>
       </c>
@@ -2349,7 +2387,7 @@
         <v>43635</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>1949</v>
       </c>
@@ -2369,7 +2407,7 @@
         <v>44416</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>1311</v>
       </c>
@@ -2389,7 +2427,7 @@
         <v>43958</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>1906</v>
       </c>
@@ -2409,7 +2447,7 @@
         <v>44107</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>1656</v>
       </c>
@@ -2429,7 +2467,7 @@
         <v>44338</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>1907</v>
       </c>
@@ -2449,7 +2487,7 @@
         <v>44455</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>1724</v>
       </c>
@@ -2469,7 +2507,7 @@
         <v>43989</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>1301</v>
       </c>
@@ -2489,7 +2527,7 @@
         <v>43990</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>1292</v>
       </c>
@@ -2509,7 +2547,7 @@
         <v>44350</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>1167</v>
       </c>
@@ -2529,7 +2567,7 @@
         <v>44489</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>1950</v>
       </c>
@@ -2549,7 +2587,7 @@
         <v>44498</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>1792</v>
       </c>
@@ -2569,7 +2607,7 @@
         <v>44376</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>1977</v>
       </c>
@@ -2589,7 +2627,7 @@
         <v>43469</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>1067</v>
       </c>
@@ -2609,7 +2647,7 @@
         <v>44168</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>1976</v>
       </c>
@@ -2629,7 +2667,7 @@
         <v>43878</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>1168</v>
       </c>
@@ -2649,7 +2687,7 @@
         <v>43805</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>1815</v>
       </c>
@@ -2669,7 +2707,7 @@
         <v>43905</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>1068</v>
       </c>
@@ -2689,7 +2727,7 @@
         <v>43500</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>1012</v>
       </c>
@@ -2709,7 +2747,7 @@
         <v>43687</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>1301</v>
       </c>
@@ -2729,7 +2767,7 @@
         <v>44181</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>1556</v>
       </c>
@@ -2749,7 +2787,7 @@
         <v>44441</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>1933</v>
       </c>
@@ -2769,7 +2807,7 @@
         <v>44455</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>1333</v>
       </c>
@@ -2789,7 +2827,7 @@
         <v>44382</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>1510</v>
       </c>
@@ -2809,7 +2847,7 @@
         <v>44133</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>1574</v>
       </c>
@@ -2829,7 +2867,7 @@
         <v>43604</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>1360</v>
       </c>
@@ -2849,7 +2887,7 @@
         <v>43701</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>1293</v>
       </c>
@@ -2869,7 +2907,7 @@
         <v>43933</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>1329</v>
       </c>
@@ -2889,7 +2927,7 @@
         <v>43568</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>1572</v>
       </c>
@@ -2909,7 +2947,7 @@
         <v>43968</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>1300</v>
       </c>
@@ -2929,7 +2967,7 @@
         <v>43902</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>1557</v>
       </c>
@@ -2949,7 +2987,7 @@
         <v>44241</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>1169</v>
       </c>
@@ -2969,7 +3007,7 @@
         <v>43704</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>1758</v>
       </c>
@@ -2989,7 +3027,7 @@
         <v>44140</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>1310</v>
       </c>
@@ -3009,7 +3047,7 @@
         <v>43740</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>1041</v>
       </c>
@@ -3029,7 +3067,7 @@
         <v>44012</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>1361</v>
       </c>
@@ -3049,7 +3087,7 @@
         <v>44304</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>1793</v>
       </c>
@@ -3069,7 +3107,7 @@
         <v>44445</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>1967</v>
       </c>
@@ -3089,7 +3127,7 @@
         <v>44436</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>1725</v>
       </c>
@@ -3109,7 +3147,7 @@
         <v>43555</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>1969</v>
       </c>
@@ -3129,7 +3167,7 @@
         <v>44274</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>1962</v>
       </c>
@@ -3149,7 +3187,7 @@
         <v>44424</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>1967</v>
       </c>
@@ -3169,7 +3207,7 @@
         <v>44480</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>1426</v>
       </c>
@@ -3189,7 +3227,7 @@
         <v>44254</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>1509</v>
       </c>
@@ -3209,7 +3247,7 @@
         <v>43840</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>1673</v>
       </c>
@@ -3229,7 +3267,7 @@
         <v>44375</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>1352</v>
       </c>
@@ -3249,7 +3287,7 @@
         <v>43792</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>1922</v>
       </c>
@@ -3269,7 +3307,7 @@
         <v>44490</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>1518</v>
       </c>
@@ -3289,7 +3327,7 @@
         <v>43867</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>1331</v>
       </c>
@@ -3309,7 +3347,7 @@
         <v>43497</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>1303</v>
       </c>
@@ -3329,7 +3367,7 @@
         <v>43487</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>1302</v>
       </c>
@@ -3349,7 +3387,7 @@
         <v>44209</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>1334</v>
       </c>
@@ -3369,7 +3407,7 @@
         <v>44401</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>1975</v>
       </c>
@@ -3389,7 +3427,7 @@
         <v>43927</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>1759</v>
       </c>
@@ -3409,7 +3447,7 @@
         <v>44379</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>1055</v>
       </c>
@@ -3429,7 +3467,7 @@
         <v>43598</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>1054</v>
       </c>
@@ -3449,7 +3487,7 @@
         <v>43973</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>1075</v>
       </c>
@@ -3469,7 +3507,7 @@
         <v>44204</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>1966</v>
       </c>
@@ -3489,7 +3527,7 @@
         <v>44376</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>1354</v>
       </c>
@@ -3509,7 +3547,7 @@
         <v>44304</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>1696</v>
       </c>
@@ -3529,7 +3567,7 @@
         <v>44355</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>1299</v>
       </c>
@@ -3549,7 +3587,7 @@
         <v>43798</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>1529</v>
       </c>
@@ -3569,7 +3607,7 @@
         <v>43896</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>1080</v>
       </c>
@@ -3589,7 +3627,7 @@
         <v>43933</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>1353</v>
       </c>
@@ -3609,7 +3647,7 @@
         <v>43475</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>1369</v>
       </c>
@@ -3629,7 +3667,7 @@
         <v>43868</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>1370</v>
       </c>
@@ -3649,7 +3687,7 @@
         <v>43715</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>1677</v>
       </c>
@@ -3669,7 +3707,7 @@
         <v>43614</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>1427</v>
       </c>
@@ -3692,5 +3730,8 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>